<commit_message>
Fix trends sheet formatting: fill blanks with em-dash, add title spacer row
- Blank year cells now show '—' instead of empty
- Title/subtitle merged across width, spacer row before blue header
- Header row properly styled with blue background (was unstyled before)
- Chart data handles NaN values, charts positioned below data table
</commit_message>
<xml_diff>
--- a/DE_ZCTA_County_Analysis.xlsx
+++ b/DE_ZCTA_County_Analysis.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -146,6 +146,9 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -265,12 +268,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$26:$D$26</f>
+              <f>'PLACES_Trends_Summary'!$E$26:$G$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$27:$D$27</f>
+              <f>'PLACES_Trends_Summary'!$E$27:$G$27</f>
             </numRef>
           </val>
         </ser>
@@ -382,12 +385,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$26:$D$26</f>
+              <f>'PLACES_Trends_Summary'!$E$26:$G$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$28:$D$28</f>
+              <f>'PLACES_Trends_Summary'!$E$28:$G$28</f>
             </numRef>
           </val>
         </ser>
@@ -499,12 +502,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$26:$D$26</f>
+              <f>'PLACES_Trends_Summary'!$E$26:$G$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$29:$D$29</f>
+              <f>'PLACES_Trends_Summary'!$E$29:$G$29</f>
             </numRef>
           </val>
         </ser>
@@ -616,12 +619,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$26:$D$26</f>
+              <f>'PLACES_Trends_Summary'!$E$26:$G$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$30:$D$30</f>
+              <f>'PLACES_Trends_Summary'!$E$30:$G$30</f>
             </numRef>
           </val>
         </ser>
@@ -733,12 +736,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$26:$D$26</f>
+              <f>'PLACES_Trends_Summary'!$E$26:$G$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$31:$D$31</f>
+              <f>'PLACES_Trends_Summary'!$E$31:$G$31</f>
             </numRef>
           </val>
         </ser>
@@ -850,12 +853,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$26:$D$26</f>
+              <f>'PLACES_Trends_Summary'!$E$26:$G$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'PLACES_Trends_Summary'!$B$32:$D$32</f>
+              <f>'PLACES_Trends_Summary'!$E$32:$G$32</f>
             </numRef>
           </val>
         </ser>
@@ -930,7 +933,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>4</row>
+      <row>24</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2520000"/>
@@ -952,7 +955,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>22</row>
+      <row>42</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2520000"/>
@@ -974,7 +977,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>40</row>
+      <row>60</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2520000"/>
@@ -996,7 +999,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>58</row>
+      <row>78</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2520000"/>
@@ -1018,7 +1021,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>76</row>
+      <row>96</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2520000"/>
@@ -1040,7 +1043,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>94</row>
+      <row>114</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5400000" cy="2520000"/>
@@ -86526,7 +86529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -86543,81 +86546,67 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Measure</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Years Covered</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Start Value (%)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>End Value (%)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>2021 Avg (%)</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>2022 Avg (%)</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>2023 Avg (%)</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Total Change (pp)</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Pct Change (%)</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Slope / Year (pp)</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Trend Direction</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>ZCTAs with Data</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -86636,8 +86625,10 @@
       <c r="D5" s="22" t="n">
         <v>27.23</v>
       </c>
-      <c r="E5" s="22" t="n">
-        <v/>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F5" s="22" t="n">
         <v>24.09</v>
@@ -86680,8 +86671,10 @@
       <c r="D6" s="22" t="n">
         <v>81.06999999999999</v>
       </c>
-      <c r="E6" s="22" t="n">
-        <v/>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F6" s="22" t="n">
         <v>78.92</v>
@@ -86727,8 +86720,10 @@
       <c r="E7" s="22" t="n">
         <v>36.41</v>
       </c>
-      <c r="F7" s="22" t="n">
-        <v/>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G7" s="22" t="n">
         <v>38.14</v>
@@ -86768,8 +86763,10 @@
       <c r="D8" s="22" t="n">
         <v>19.05</v>
       </c>
-      <c r="E8" s="22" t="n">
-        <v/>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F8" s="22" t="n">
         <v>17.35</v>
@@ -86812,8 +86809,10 @@
       <c r="D9" s="22" t="n">
         <v>35.4</v>
       </c>
-      <c r="E9" s="22" t="n">
-        <v/>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F9" s="22" t="n">
         <v>37.09</v>
@@ -86856,8 +86855,10 @@
       <c r="D10" s="22" t="n">
         <v>13.08</v>
       </c>
-      <c r="E10" s="22" t="n">
-        <v/>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F10" s="22" t="n">
         <v>14.53</v>
@@ -86900,8 +86901,10 @@
       <c r="D11" s="22" t="n">
         <v>21.93</v>
       </c>
-      <c r="E11" s="22" t="n">
-        <v/>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F11" s="22" t="n">
         <v>20.49</v>
@@ -86944,8 +86947,10 @@
       <c r="D12" s="22" t="n">
         <v>14.24</v>
       </c>
-      <c r="E12" s="22" t="n">
-        <v/>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F12" s="22" t="n">
         <v>15.23</v>
@@ -86988,8 +86993,10 @@
       <c r="D13" s="22" t="n">
         <v>11.18</v>
       </c>
-      <c r="E13" s="22" t="n">
-        <v/>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F13" s="22" t="n">
         <v>11.8</v>
@@ -87032,8 +87039,10 @@
       <c r="D14" s="22" t="n">
         <v>15.85</v>
       </c>
-      <c r="E14" s="22" t="n">
-        <v/>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F14" s="22" t="n">
         <v>15.37</v>
@@ -87076,8 +87085,10 @@
       <c r="D15" s="22" t="n">
         <v>7.09</v>
       </c>
-      <c r="E15" s="22" t="n">
-        <v/>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F15" s="22" t="n">
         <v>7.45</v>
@@ -87120,8 +87131,10 @@
       <c r="D16" s="22" t="n">
         <v>7.52</v>
       </c>
-      <c r="E16" s="22" t="n">
-        <v/>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F16" s="22" t="n">
         <v>7.86</v>
@@ -87167,8 +87180,10 @@
       <c r="E17" s="22" t="n">
         <v>87.63</v>
       </c>
-      <c r="F17" s="22" t="n">
-        <v/>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G17" s="22" t="n">
         <v>87.34</v>
@@ -87208,8 +87223,10 @@
       <c r="D18" s="22" t="n">
         <v>13.83</v>
       </c>
-      <c r="E18" s="22" t="n">
-        <v/>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F18" s="22" t="n">
         <v>13.57</v>
@@ -87252,8 +87269,10 @@
       <c r="D19" s="22" t="n">
         <v>3.74</v>
       </c>
-      <c r="E19" s="22" t="n">
-        <v/>
+      <c r="E19" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F19" s="22" t="n">
         <v>3.92</v>
@@ -87296,8 +87315,10 @@
       <c r="D20" s="22" t="n">
         <v>12.79</v>
       </c>
-      <c r="E20" s="22" t="n">
-        <v/>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F20" s="22" t="n">
         <v>12.93</v>
@@ -87340,8 +87361,10 @@
       <c r="D21" s="22" t="n">
         <v>8.890000000000001</v>
       </c>
-      <c r="E21" s="22" t="n">
-        <v/>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F21" s="22" t="n">
         <v>8.75</v>
@@ -87384,8 +87407,10 @@
       <c r="D22" s="22" t="n">
         <v>11.08</v>
       </c>
-      <c r="E22" s="22" t="n">
-        <v/>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F22" s="22" t="n">
         <v>11.01</v>
@@ -87446,9 +87471,7 @@
           <t>Physical Inactivity %</t>
         </is>
       </c>
-      <c r="B27" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B27" s="22" t="n"/>
       <c r="C27" s="22" t="n">
         <v>24.09</v>
       </c>
@@ -87462,9 +87485,7 @@
           <t>Routine Checkup %</t>
         </is>
       </c>
-      <c r="B28" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B28" s="22" t="n"/>
       <c r="C28" s="22" t="n">
         <v>78.92</v>
       </c>
@@ -87481,9 +87502,7 @@
       <c r="B29" s="22" t="n">
         <v>36.41</v>
       </c>
-      <c r="C29" s="22" t="n">
-        <v/>
-      </c>
+      <c r="C29" s="22" t="n"/>
       <c r="D29" s="22" t="n">
         <v>38.14</v>
       </c>
@@ -87494,9 +87513,7 @@
           <t>Fair/Poor Health %</t>
         </is>
       </c>
-      <c r="B30" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B30" s="22" t="n"/>
       <c r="C30" s="22" t="n">
         <v>17.35</v>
       </c>
@@ -87510,9 +87527,7 @@
           <t>Obesity %</t>
         </is>
       </c>
-      <c r="B31" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B31" s="22" t="n"/>
       <c r="C31" s="22" t="n">
         <v>37.09</v>
       </c>
@@ -87526,9 +87541,7 @@
           <t>Current Smoking %</t>
         </is>
       </c>
-      <c r="B32" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B32" s="22" t="n"/>
       <c r="C32" s="22" t="n">
         <v>14.53</v>
       </c>
@@ -87542,9 +87555,7 @@
           <t>Depression %</t>
         </is>
       </c>
-      <c r="B33" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B33" s="22" t="n"/>
       <c r="C33" s="22" t="n">
         <v>20.49</v>
       </c>
@@ -87558,9 +87569,7 @@
           <t>Binge Drinking %</t>
         </is>
       </c>
-      <c r="B34" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B34" s="22" t="n"/>
       <c r="C34" s="22" t="n">
         <v>15.23</v>
       </c>
@@ -87574,9 +87583,7 @@
           <t>Housing Insecurity %</t>
         </is>
       </c>
-      <c r="B35" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B35" s="22" t="n"/>
       <c r="C35" s="22" t="n">
         <v>11.8</v>
       </c>
@@ -87590,9 +87597,7 @@
           <t>Frequent Mental Distress %</t>
         </is>
       </c>
-      <c r="B36" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B36" s="22" t="n"/>
       <c r="C36" s="22" t="n">
         <v>15.37</v>
       </c>
@@ -87606,9 +87611,7 @@
           <t>Coronary Heart Disease %</t>
         </is>
       </c>
-      <c r="B37" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B37" s="22" t="n"/>
       <c r="C37" s="22" t="n">
         <v>7.45</v>
       </c>
@@ -87622,9 +87625,7 @@
           <t>COPD %</t>
         </is>
       </c>
-      <c r="B38" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B38" s="22" t="n"/>
       <c r="C38" s="22" t="n">
         <v>7.86</v>
       </c>
@@ -87641,9 +87642,7 @@
       <c r="B39" s="22" t="n">
         <v>87.63</v>
       </c>
-      <c r="C39" s="22" t="n">
-        <v/>
-      </c>
+      <c r="C39" s="22" t="n"/>
       <c r="D39" s="22" t="n">
         <v>87.34</v>
       </c>
@@ -87654,9 +87653,7 @@
           <t>Food Insecurity %</t>
         </is>
       </c>
-      <c r="B40" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B40" s="22" t="n"/>
       <c r="C40" s="22" t="n">
         <v>13.57</v>
       </c>
@@ -87670,9 +87667,7 @@
           <t>Stroke %</t>
         </is>
       </c>
-      <c r="B41" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B41" s="22" t="n"/>
       <c r="C41" s="22" t="n">
         <v>3.92</v>
       </c>
@@ -87686,9 +87681,7 @@
           <t>Diabetes %</t>
         </is>
       </c>
-      <c r="B42" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B42" s="22" t="n"/>
       <c r="C42" s="22" t="n">
         <v>12.93</v>
       </c>
@@ -87702,9 +87695,7 @@
           <t>Uninsured 18-64 %</t>
         </is>
       </c>
-      <c r="B43" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B43" s="22" t="n"/>
       <c r="C43" s="22" t="n">
         <v>8.75</v>
       </c>
@@ -87718,9 +87709,7 @@
           <t>Current Asthma %</t>
         </is>
       </c>
-      <c r="B44" s="22" t="n">
-        <v/>
-      </c>
+      <c r="B44" s="22" t="n"/>
       <c r="C44" s="22" t="n">
         <v>11.01</v>
       </c>
@@ -87729,6 +87718,10 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>